<commit_message>
Update product import template instructions for six photos
</commit_message>
<xml_diff>
--- a/public/product-import-template.xlsx
+++ b/public/product-import-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R855ce8d3606b4742"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="2" r:id="R094dcd4c5a0747aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R41bf3db3395f40a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="2" r:id="R224e306c4ee64682"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2158,10 +2158,10 @@
         <x:v>Photos</x:v>
       </x:c>
       <x:c r="B19" s="9" t="str">
-        <x:v>Excel mein photos nahi. Import ke baad Admin &gt; Listings &gt; Edit se 4 photos add karein.</x:v>
+        <x:v>Excel mein photos nahi. Import ke baad Admin &gt; Listings &gt; Edit se 6 photos add karein.</x:v>
       </x:c>
       <x:c r="C19" s="9" t="str">
-        <x:v>Main, hover, extra 3, extra 4</x:v>
+        <x:v>Main, hover, extra 3, 4, 5, 6</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="34" customHeight="1">

</xml_diff>